<commit_message>
research: Teams Counted moved to column C in all workbooks (was buried at far right)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/research/provinces/SportsHub-New-Brunswick.xlsx
+++ b/docs/research/provinces/SportsHub-New-Brunswick.xlsx
@@ -441,7 +441,7 @@
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
@@ -471,77 +471,77 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Teams Counted</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Owner/Principal</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Programs</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Leagues</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Software</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
-        </is>
-      </c>
-      <c r="Q1" s="2" t="inlineStr">
-        <is>
-          <t>Teams Counted</t>
         </is>
       </c>
     </row>
@@ -556,57 +556,57 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Chaleur (BNB North)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Bathurst</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>(506) 543-1642</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>colin.brewster@holliswealth.com</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>https://www.bathurstminorbasketball.ca/</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Nonprofit teaching youth of the Chaleur region; season October to end of March across 5 divisions; summer skills day camp; rep teams compete as the 'Bathurst Blazers'</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>BNB Provincial League (U12-U14); Bathurst Minor Basketball house divisions (own program)</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>reported</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>https://www.bathurstminorbasketball.ca/</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Website (including /en/executive page) returned HTTP 500 on every fetch at check — contacts pulled from search snippets: second contact david.chaisson@nbed.nb.ca; roles for Brewster/Chaisson unconfirmed. Bilingual Chaleur market. No youth basketball club found further north in Campbellton/Dalhousie/Restigouche — BNB North region has only 3 member entries total. | Also listed as: Bathurst Minor Basketball Association</t>
         </is>
@@ -623,62 +623,62 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Dieppe</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>76 rue Emmanuel Street, Dieppe, NB E1A 2J5</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>506-857-3807 ext. 113</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>programmer@dbgc.org</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>https://bgcdieppe.ca/programs/drop-in/</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Monday-night youth basketball program ages 7-18 (6:30-8:00pm, academic year), delivered with Maritime Progression; $10 annual membership</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>multi-sport org (youth club charity)</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Microsoft Forms (program registration)</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>https://bgcdieppe.ca/programs/drop-in/</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Drop-in programming only, no teams; outsources coaching to Maritime Progression.</t>
         </is>
@@ -695,62 +695,62 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Dieppe</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>presidence@basketballdieppe.ca</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>https://basketballdieppe.ca/</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Pierre Duguay-Boudreau, directeur général / founding leader (per 2021 Radio-Canada launch coverage)</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Francophone recreational + competitive development, launched Aug 2021 for ages 6-14 (entirely in French); Saison d'hiver (winter league), camps d'été, ligue adulte; affordability mandate</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Basketball Dieppe winter season (Saison d'hiver) — operator; BNB Provincial League (U12-U14)</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>community nonprofit (first fully francophone basketball association in NB)</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>TeamSnap (registration form go.teamsnap.com/forms/429947, 'Basketball Dieppe Inc.'); GoDaddy Website Builder site</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>https://basketballdieppe.ca/</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Contact page is a web form only — no published email/phone. Serves the Acadian francophone community; a Village de Memramcook page has referenced Basketball Dieppe for Memramcook youth (page now 404), suggesting catchment beyond Dieppe.</t>
         </is>
@@ -767,48 +767,48 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>Carleton County (north)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Florenceville-Bristol</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>https://www.facebook.com/share/1CY9UV55im/?mibextid=wwXIfr</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Youth minor basketball serving Carleton North communities (Florenceville-Bristol, Centreville, Bath)</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>primary</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>BNB 2025-26 member (Central/West Region); Facebook-only presence.</t>
         </is>
-      </c>
-      <c r="Q5" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -822,47 +822,47 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Capital region (BNB Central/West)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Fredericton</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>https://www.facebook.com/p/Fredericton-Jr-Freeze-Girls-Basketball-Team-61574570303956/</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Charlene Woolaver, Head Coach</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Girls basketball for players entering Grades 9-11; spring play beginning 2025; created to close the participation gap after BNB's age 5-14 system; wears Fredericton Freeze (MWBA) colours</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>community nonprofit (youth arm of MWBA Fredericton Freeze)</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>primary</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>https://themwba.ca/2025/03/24/junior-freeze-becomes-reality/</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>Listed as 'Jr. Freeze' on BNB registry (Central/West). Program 'falls under Basketball New Brunswick's umbrella' per MWBA announcement. | enriched 2026-07-18</t>
         </is>
@@ -879,68 +879,68 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" t="n">
+        <v>28</v>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>Fredericton</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Fredericton</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>info@frederictonfusion.com</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>https://www.frederictonfusion.com/</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Dr. Jonathon Edwards, co-founder &amp; President (UNB kinesiology assistant dean; president as of 2024 UNB profile)</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Fusion City League (recreational house league, U11/U12/U13-14 boys &amp; girls); competitive/rep teams (e.g., U16 boys); Jr. NBA; summer skills clinics U11-U14; junior referee program; hosts annual Winter Classic tournament (50+ teams from Atlantic Canada); 700+ players</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Fusion City League (Fredericton Youth Basketball Association); BNB Provincial League (U12-U14); BNB-sanctioned club tournament circuit (winter weekends); BNB Provincial Championships U12/U13/U14</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>RAMP InterActive (website + registration) AND TeamLinkt (league operations site leagues.teamlinkt.com/fybafrederictonfusion)</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>https://www.frederictonfusion.com/</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>Formed 2020 by merging two rival clubs: YMCA Competitive Basketball Club (YCBC) Capitals and Northside Minor Basketball Association (NMBA) Lions — both now legacy. Grew participation from 200 to 700+. Secondary email frederictonbasketball@outlook.com. Dual RAMP+TeamLinkt stack is notable competitive intel.</t>
         </is>
-      </c>
-      <c r="Q7" t="n">
-        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -954,52 +954,52 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Fredericton</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Fredericton</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>https://themwba.ca/2025/03/24/junior-freeze-becomes-reality/</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Charlene Woolaver, Head Coach (former UNB Reds star); program launched by the Fredericton Freeze (MWBA)</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Girls spring team for players entering Grades 9-11; fills gap in teenage girls' basketball; wears Freeze colours; under Basketball NB umbrella</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>BNB-sanctioned spring play (under Basketball NB umbrella)</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>community program of semi-pro women's team (Fredericton Freeze, MWBA)</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>reported</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>https://themwba.ca/2025/03/24/junior-freeze-becomes-reality/</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>Listed as 'Jr. Freeze' on BNB 2025-26 member list (Central/West Region). First season spring 2025.</t>
         </is>
@@ -1016,72 +1016,72 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Fredericton</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Fredericton</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>UNB Fredericton campus (Currie Center), Fredericton, NB</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>(506) 453-4579</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>redsrec@unb.ca</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>https://goredsgo.ca/sports/wbkb/junior_basketball</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Jeff Speedy, founder (UNB Director of Athletics, former UNB Reds women's head coach)</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Girls spring/early-summer club basketball in four age classes (U11, U12, U13, U14); ~16 games/season, 2-3 practices weekly; hosts 'UNB School's Out Shootout' each June; scholarships available; coached by UNB players/alumni</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>BNB-sanctioned spring league/tournament play (regional)</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>university-affiliated youth club program</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>UNB Recreation Services online registration portal (recreation.unbf.ca)</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>https://goredsgo.ca/sports/wbkb/junior_basketball</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>Listed as 'Junior Reds' on BNB 2025-26 member list (Central/West Region). | enriched 2026-07-18</t>
         </is>
@@ -1098,72 +1098,72 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Fredericton</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Fredericton</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>UNB Fredericton campus (Currie Center), Fredericton, NB</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>(506) 453-4579</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>redsyouth@unb.ca</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>https://goredsgo.ca/sports/mbkb/2021-22/releases/springleagues</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Joe Salerno, founder (UNB Reds men's basketball head coach)</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Competitive select club program for advanced boys (launched 2022 with U14 team via two-day tryout); exhibition games and regional tournaments; players train alongside UNB men's program</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>BNB-sanctioned club tournament circuit (winter weekends)</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>university-affiliated youth club program</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>UNB Recreation Services online registration portal (recreation.unbf.ca)</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>reported</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>https://goredsgo.ca/sports/mbkb/2021-22/releases/springleagues</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>Listed as 'Reds Selects' on BNB 2025-26 member list; program details are from 2022 launch coverage and may have evolved. | enriched 2026-07-18</t>
         </is>
@@ -1180,67 +1180,67 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Capital region (BNB Central/West)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Fredericton</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Richard J. Currie Center, University of New Brunswick, Fredericton</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>(506) 453-4579</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>redsyouth@unb.ca</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>https://goredsgo.ca/sports/wbkb/junior_basketball</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Jeff Speedy, Director of Athletics</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>University-run youth club programs: Junior Reds girls spring/early-summer teams U11, U12, U13, U14; Jr. Reds boys spring league U10, U12, U14; REDS Select — advanced U14 boys team chosen by two-day tryout, playing regional exhibitions and tournaments; REDS girls basketball camps</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>university-operated youth club program (listed on BNB registry as two entries: 'Junior Reds' and 'Reds Selects')</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>UNB Recreation Services online portal (recreation.unbf.ca)</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>https://goredsgo.ca/sports/wbkb/junior_basketball</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>Operated by UNB REDS Athletics/Recreation (varsity-affiliated but a registered BNB youth club program, not school-board basketball). UNB partners with Fredericton Fusion (coaches on Fusion board). | enriched 2026-07-18</t>
         </is>
@@ -1257,67 +1257,67 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Fredericton</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Fredericton</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>231 Mataya Drive, Fredericton, NB</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>yfc.elite.basketball@gmail.com</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>https://www.yfc-elite-basketball-association.ca/</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>Matthew Raiche, President</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>Grassroots family-driven association; skill development and competitive play; U18 boys program (Nov-Apr) for high-school-aged players; volunteer coaches</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>BNB-sanctioned club play (Looking for Games circuit); BNB-sanctioned club tournament circuit (winter weekends); BNB Age Class Provincials (U16 &amp; U18)</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>RAMP (registrations) + TeamLinkt (club page leagues.teamlinkt.com)</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>https://www.yfc-elite-basketball-association.ca/</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>President Matthew Raiche confirmed in CBC News article (quoted as YFC Elite president). Address from Facebook/local listings.</t>
         </is>
@@ -1334,62 +1334,62 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Capital region</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Fredericton</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>570 York Street, Fredericton, NB E3B 3R3</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>(506) 462-3000 ext. 0</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>info@ymcafredericton.org</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>https://fredericton.ymca.ca/programs/youth-registered-programs-gr-1-8/youth-basketball/</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Jr. NBA developmental skills program (partnership with Canada Basketball and the NBA) in six age groups, ages 5-16; Sept-Mar season, ~$55/participant; sessions at YMCA gym and Priestman St &amp; Connaught St schools</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>multi-sport org (YMCA charity)</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>ActiveNet / Active Communities registration portal (anc.ca.apm.activecommunities.com)</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>https://fredericton.ymca.ca/programs/youth-registered-programs-gr-1-8/youth-basketball/</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>The YMCA's former competitive club, YCBC Capitals (host of the Holiday Hoops Classic, once eastern Canada's largest youth tournament), merged into Fredericton Fusion in 2020 — YMCA now runs rec/skills only.</t>
         </is>
@@ -1406,57 +1406,57 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Multiple NB regions incl. Fredericton, upper river valley, and northwest</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Fredericton / Woodstock / Edmundston (HQ Moncton)</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>506-380-2255</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>sweatacademy@gmail.com</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>https://www.sweatacademy.com/</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Serge Langis, co-owner (former pro player; also coaching basketball revival at Cité des Jeunes d'Edmundston)</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>Elite off-season player development (basketball + baseball): intensive training, spring sessions, game-simulated drills for youth and high school athletes; branches: Capital City (Fredericton), Western Valley (Woodstock), Madawaska-Victoria (Edmundston), plus Moncton</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>private academy (multi-sport, for-profit)</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>https://www.sweatacademy.com/</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>Only basketball organization listed in the City of Edmundston recreation directory — no community minor basketball association found in Edmundston or Campbellton (BNB North Region lists only Miramichi, Acadie, Bathurst). Basketball in Edmundston is otherwise school-based (Cité des Jeunes, coach Serge Langis, per CIMT-CHAU news).</t>
         </is>
@@ -1473,62 +1473,62 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Saint John area</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Grand Bay-Westfield</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>(506) 738-1086</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>https://rvba.ca/</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>Keith Thomas, President</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>House league (Puppy U7, U9, U11, U14); rep teams U11/U13/U14 (October tryouts); spring league Apr-Jun (8 weeks, in-house scrimmages); 30+ years operating</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>RVBA house league (Grand Bay-Westfield); RVBA Spring League; BNB Provincial Championships U12/U13/U14; BNB-sanctioned club tournament circuit (winter weekends)</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>TeamSnap (registration/app)</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>https://rvba.ca/</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>Full board published: VP Emily Thomas, Secretary Barb Thomas, Treasurer Kenzie London + 6 directors. Distinct from Riverview MBA (Moncton area).</t>
         </is>
@@ -1545,37 +1545,37 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Victoria County / Northwest (BNB Central/West)</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Grand Falls (Grand-Sault)</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>Youth minor basketball</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>uncertain</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
+      <c r="Q16" t="inlineStr">
         <is>
           <t>BNB registry entry only; no website/social found. This is the nearest BNB member club to Edmundston — NO BNB member club exists in Edmundston itself; the only Edmundston youth basketball found is a school-based program at Cité des Jeunes led by Serge Langis (cimtchau.ca news), excluded as school basketball.</t>
         </is>
@@ -1592,68 +1592,68 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
         <is>
           <t>Saint John area (Kings County)</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Hampton</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>hamptonminorbasketball@gmail.com</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>https://hamptonminorbasketball.com/</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="J17" t="inlineStr">
         <is>
           <t>David Turner, President (2026/27 board)</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>Volunteer-run not-for-profit community basketball for youth U5-U14 (house league)</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>Hampton Minor Basketball Association house league</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>RAMP InterActive (current website); TeamSnap (registration form go.teamsnap.com/forms/283797; legacy TeamSnap Sites page); legacy Pointstreak Sites website</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr">
+      <c r="O17" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>https://hamptonminorbasketball.com/</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr">
+      <c r="Q17" t="inlineStr">
         <is>
           <t>Board 2026/27: VP Bradford Rogers, Treasurer Doug Nutter, Secretary Candace Muir, Coach Director Luke Johnson, Officials Director Alex Richard. Migrated Pointstreak → TeamSnap → RAMP (competitive-intel: three platforms in site history).</t>
         </is>
-      </c>
-      <c r="Q17" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1667,42 +1667,42 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Carleton County (BNB Central/West)</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Hartland</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/222366587892722/</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>Youth basketball in the Hartland area; Steve Nash mini program for K-3 (late-Oct registration, Tuesday-evening sessions) per Town of Hartland recreation listings; uses Central Carleton Community Complex</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr">
+      <c r="O18" t="inlineStr">
         <is>
           <t>reported</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="P18" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr">
+      <c r="Q18" t="inlineStr">
         <is>
           <t>Facebook group is the primary presence. | Also listed as: Central Carleton Basketball Association</t>
         </is>
@@ -1719,42 +1719,42 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>York County (rural Fredericton area)</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Harvey Station</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/390133675984191/</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>Youth minor basketball</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr">
+      <c r="O19" t="inlineStr">
         <is>
           <t>primary</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="P19" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
+      <c r="Q19" t="inlineStr">
         <is>
           <t>BNB 2025-26 member (Central/West Region); Facebook group is only online presence found. Harvey is a strong basketball town at high-school level.</t>
         </is>
@@ -1771,57 +1771,57 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>York County (southwest)</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>McAdam</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>146 Saunders Road, McAdam, NB E6J 1L2</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>506-784-1422</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>mcadamminorbasketball@outlook.com</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>https://www.facebook.com/mcadambasketball</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>Youth minor basketball (village has two gymnasiums used for programs)</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr">
+      <c r="O20" t="inlineStr">
         <is>
           <t>primary</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="P20" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr">
+      <c r="Q20" t="inlineStr">
         <is>
           <t>BNB 2025-26 member (Central/West Region); Facebook is only online presence found. | Community minor association (village of ~1,100); Basketball NB 2025-26 member, Central/West Region (https://www.basketball.nb.ca/content/find-a-club-association). Email extracted from their public Facebook page 'About' info (https://www.facebook.com/mcadambasketball — categorized Youth Organization, McAdam NB, 177 followers). No street address, phone, website, or named executive published. Partners with St. Stephen Minor Basketball Association for camps and events (per Facebook page posts). | enriched 2026-07-18</t>
         </is>
@@ -1838,58 +1838,58 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" t="n">
+        <v>7</v>
+      </c>
+      <c r="D21" t="inlineStr">
         <is>
           <t>Miramichi / North Shore</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Miramichi</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>https://leagues.teamlinkt.com/miramichiriverhoops</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>Youth basketball league and rep teams; registration held at MVHS Gymnasium; funds a bursary at Miramichi Valley High School</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>Miramichi River Hoops league; BNB Provincial League (U12-U14)</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>TeamLinkt (current league/site) + RAMP (registrations); formerly GOALLINE (miramichihoops.goalline.ca now redirects to Stack Sports)</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>https://leagues.teamlinkt.com/miramichiriverhoops/Schedule</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="Q21" t="inlineStr">
         <is>
           <t>TeamLinkt contact page lists a president 'Matt' but appears to be a placeholder profile (phone 0123456789) — treat as unknown. X handle @RiverHoops. Platform migration GOALLINE→TeamLinkt+RAMP is competitive intel.</t>
         </is>
-      </c>
-      <c r="Q21" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="22">
@@ -1903,47 +1903,47 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Moncton</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>https://www.facebook.com/506Shamrocks/</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>U12/U14 youth team program (Shamrocks); development stream ('Elevate') feeding 506 Elite teams</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>BNB-sanctioned club tournament circuit (winter weekends)</t>
         </is>
       </c>
-      <c r="L22" t="inlineStr">
+      <c r="M22" t="inlineStr">
         <is>
           <t>private development program</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>uncertain</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>https://www.facebook.com/506Shamrocks/</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr">
+      <c r="Q22" t="inlineStr">
         <is>
           <t>506shamrocks.com DNS is dead; Facebook page renamed '506 Elevate Basketball'. Roster described as best U14s from the 506 Elevate program plus 506 Elite tryout cuts — likely absorbed into 506 Elite's Elevate League. Kept as separate row for dedupe; verify before outreach.</t>
         </is>
@@ -1960,67 +1960,67 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB (facility in Irishtown, Greater Moncton)</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Moncton</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>2603 NB-115, Irishtown, NB E1H 2M5 (Maple Hills / Moncton Kia Centre)</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>(506) 378-2880</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>https://506elite.com/</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="J23" t="inlineStr">
         <is>
           <t>Nate Horsman, Managing Partner of TH Sports Group &amp; 506 Elite</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>Elevate League U7-U18 (in-house developmental league); Elite Teams U11-U17 (selective travel teams); Elite Academy U15-U18 (full-time academics + high-performance training); Nike Sports Camps (basketball, soccer, multi-sport); 506 Shamrocks U12/U14 program (top Elevate players + non-Elite-team players); also pickleball/teeball programming</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>506 Elite 'Elevate League' (U7-U18) — operator; BNB-sanctioned club tournament circuit (winter weekends); BNB Provincial League (U12-U14); BNB Provincial Championships U12/U13/U14</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
+      <c r="M23" t="inlineStr">
         <is>
           <t>private academy / for-profit multi-sport facility</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>TeamLinkt (league site leagues.teamlinkt.com/506elitebasketball) + RAMP Registrations (program enrollment) + Citrus Camps (Nike camps via Sports Camps Canada)</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr">
+      <c r="O23" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>https://506elite.com/</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr">
+      <c r="Q23" t="inlineStr">
         <is>
           <t>BNB member. Uses BOTH TeamLinkt and RAMP — dual competitive-intel signal. Also fields an adult team in BNB's NB Mens League (out of youth scope). 506 Elevate Basketball / 506 Shamrocks brands fold into this org.</t>
         </is>
@@ -2037,62 +2037,62 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>Moncton</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>506-304-6982</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>orlandopalmer@live.ca</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>https://maritimeprogression.com/</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="J24" t="inlineStr">
         <is>
           <t>Orlando Palmer, founder/lead trainer</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>Youth basketball training sessions Oct-Apr (Fridays at Champlain School, weekends at CEPS Louis-J.-Robichaud, U de Moncton) $60/session; 1-on-1 personal training $100/session; summer camps</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="M24" t="inlineStr">
         <is>
           <t>private academy / training business</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>Own website booking/e-commerce (maritimeprogression.com/product/book-now/)</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="O24" t="inlineStr">
         <is>
           <t>primary</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="P24" t="inlineStr">
         <is>
           <t>https://maritimeprogression.com/</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="Q24" t="inlineStr">
         <is>
           <t>Not on BNB club registry (training service, no registered teams found).</t>
         </is>
@@ -2109,78 +2109,78 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" t="n">
+        <v>45</v>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>Moncton</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>96 Norwood Avenue, Suite #301, Moncton, NB E1C 6L9</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>(506) 295-5588</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>executivedirector@monctonbasketball.ca</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>https://www.monctonbasketball.ca/</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>Peter Graves, President (board also: Nick Robichaud VP, Simone Hanham Secretary, Richard Walker Treasurer, Roberto DiDonato Past President; staffed Executive Director role, name not published)</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>Recreational house leagues U7, U9, U11, U14, U18 (fall + spring seasons); competitive 'Provincial Program' rep teams (Moncton Hawks, Gold/Black tiers from U11 up); Hawks summer camps</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>Moncton Basketball Association (MBA) recreational league; MBA spring league; BNB Provincial League (U12-U14); BNB Provincial Championships U12/U13/U14; BNB U11 Kickoff (Nov) &amp; U11 Spring Finale (Feb); BNB Age Class Provincials (U16 &amp; U18); BNB-sanctioned club tournament circuit; Moncton Basketball Association (MBA) recreational + spring leagues; BNB-sanctioned club tournament circuit (winter weekends)</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>RAMP InterActive (website, registrations, official assigning, RAMP Team App)</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
+      <c r="P25" t="inlineStr">
         <is>
           <t>https://www.monctonbasketball.ca/</t>
         </is>
       </c>
-      <c r="P25" t="inlineStr">
+      <c r="Q25" t="inlineStr">
         <is>
           <t>Self-described longest-standing, most affordable association in Moncton area; successor identity to legacy Moncton Kiwanis Minor Basketball Association (MKMBA). Both monctonbasketball.ca (RAMP) and a legacy 'Basketball Moncton' WordPress presence exist. | Also listed as: Moncton Basketball Association (MBA)</t>
         </is>
-      </c>
-      <c r="Q25" t="n">
-        <v>45</v>
       </c>
     </row>
     <row r="26">
@@ -2194,72 +2194,72 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Moncton</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>120 High St., Suite 101, Moncton, NB E1C 5W1</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>(506) 384-7614</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>executivedirector@mkmba.ca</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>https://www.sportsengine.com/org/moncton-kiwanis-minor-basketball-association</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="J26" t="inlineStr">
         <is>
           <t>Dusty Tower, President</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>Legacy recreational league ('Playing for Fun and Playing Fair', est. ~1981): pre-season camp, mini camp, rec camps, competitive divisions U12/U14 boys &amp; girls; fall season late Oct-Feb</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>MKMBA - Moncton Kiwanis Minor Basketball Association recreational league (LEGACY); MKMBA - Moncton Kiwanis Minor Basketball Association (LEGACY)</t>
         </is>
       </c>
-      <c r="L26" t="inlineStr">
+      <c r="M26" t="inlineStr">
         <is>
           <t>community nonprofit (legacy)</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>Legacy stack: SportsEngine org page, Pointstreak (mkmba.hoopstats.pointstreak.com + pointstreaksites.com/view/mkmba), itSportsNet league pages</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>reported</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
+      <c r="P26" t="inlineStr">
         <is>
           <t>https://www.sportsengine.com/org/moncton-kiwanis-minor-basketball-association</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
+      <c r="Q26" t="inlineStr">
         <is>
           <t>Appears superseded by / rebranded as Moncton Basketball Association (not on current BNB club registry; MBA is). Kept as legacy row for dedupe — contact info is historical, do not treat as live. Instagram handle @mkmba1981 suggests founded 1981. | Also listed as: Moncton Kiwanis Minor Basketball Association (MKMBA) | enriched 2026-07-18</t>
         </is>
@@ -2276,67 +2276,67 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>Moncton</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>506-962-3559</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>nxtlevelbasketball@hotmail.com</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>https://nxtlevelbasketball.wixsite.com/nxtlevel</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="J27" t="inlineStr">
         <is>
           <t>Troy Mackenzie, founder/director &amp; lead instructor (est. 2013; also head coach of MWBA Moncton Mystics)</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>Private training: 1-on-1, small groups, ball handling, shot correction (shooting machine), agility/cardio; also fields youth teams in BNB competitions</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>BNB Provincial League (U12-U14)</t>
         </is>
       </c>
-      <c r="L27" t="inlineStr">
+      <c r="M27" t="inlineStr">
         <is>
           <t>private academy / training business</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>Wix (website + booking); teams administered through BNB's RAMP</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>primary</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
+      <c r="P27" t="inlineStr">
         <is>
           <t>https://nxtlevelbasketball.wixsite.com/nxtlevel</t>
         </is>
       </c>
-      <c r="P27" t="inlineStr">
+      <c r="Q27" t="inlineStr">
         <is>
           <t>Listed on BNB club registry via its Facebook group (facebook.com/groups/nxtlevelbasketball); 'committed to raising the level of basketball in Eastern New Brunswick'.</t>
         </is>
@@ -2353,57 +2353,57 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB (also Fredericton, Woodstock, Edmundston locations)</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>Moncton</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>506-380-2255</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>sweatacademy@gmail.com</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>https://www.sweatacademy.com/</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="J28" t="inlineStr">
         <is>
           <t>Serge Langis, co-owner (20+ yr coach; ex-Moncton Miracles NBL Canada head coach 2015-16)</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>Elite basketball and baseball player development; offseason/spring training sessions; targets middle school, high school and university-level athletes across 4 NB cities</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr">
+      <c r="M28" t="inlineStr">
         <is>
           <t>private academy (basketball + baseball elite development, ~8 years operating)</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>primary</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
+      <c r="P28" t="inlineStr">
         <is>
           <t>https://www.sweatacademy.com/</t>
         </is>
       </c>
-      <c r="P28" t="inlineStr">
+      <c r="Q28" t="inlineStr">
         <is>
           <t>Multi-city training business headquartered in the Moncton area; no league play — development sessions only.</t>
         </is>
@@ -2420,57 +2420,57 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB (HQ; satellite locations Fredericton, Woodstock, Edmundston)</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Moncton</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>506-380-2255</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>sweatacademy@gmail.com</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>https://www.sweatacademy.com/</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>Serge Langis, Co-Owner &amp; President (ex-Moncton Miracles NBL Canada head coach); Michael MacDougall, Co-Owner (Mount Allison Mounties men's assistant coach)</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>Elite off-season basketball (and baseball) player development; spring sessions and year-round training targeting high-school and university-level competitive players</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>private academy (for-profit)</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
+      <c r="O29" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
+      <c r="P29" t="inlineStr">
         <is>
           <t>https://www.sweatacademy.com/</t>
         </is>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="Q29" t="inlineStr">
         <is>
           <t>Training-only (no published league teams). Four NB locations branded SA Moncton / SA Capital City / SA Western Valley / SA Madawaska-Victoria; Moncton is home base — satellites belong to other regional sweeps.</t>
         </is>
@@ -2487,67 +2487,67 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>Moncton</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>30 War Veterans Ave., Moncton (YMCA Vaughan Harvey); also 70 Twin Oaks Dr. (YMCA Moncton North)</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>506-857-0606</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>info@ymcamoncton.ca</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>https://moncton.ymca.ca/programs/child-youth-programs/</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="J30" t="inlineStr">
         <is>
           <t>Zane Korytko — CEO (retiring July 31, 2026; incoming CEO Ryan Johnston starts summer 2026)</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>Youth basketball fundamentals program ages 5-12 (dribbling, shooting, passing drills + friendly games) at two branches; seasonal availability</t>
         </is>
       </c>
-      <c r="L30" t="inlineStr">
+      <c r="M30" t="inlineStr">
         <is>
           <t>multi-sport org (charitable)</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>YMCA in-house registration</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>primary</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
+      <c r="P30" t="inlineStr">
         <is>
           <t>https://moncton.ymca.ca/programs/child-youth-programs/</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
+      <c r="Q30" t="inlineStr">
         <is>
           <t>Skills program only — no teams or league play; marginal GTM target. | Nonprofit community organization (YMCA), not a rep club — runs 'Basketball Skills &amp; Drills' for ages 5-12 (source: https://moncton.ymca.ca/programs/child-youth-programs/). Second facility: YMCA Moncton North, 70 Twin Oaks Dr. Contact info source: https://moncton.ymca.ca/about-us/contact-us/. CEO transition source: https://moncton.ymca.ca/ymca-of-greater-moncton-announces-ryan-johnston-as-incoming-ceo/ and LinkedIn (Zane Korytko, CEO).</t>
         </is>
@@ -2564,47 +2564,47 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Victoria County / upper river valley</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Perth-Andover</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>https://svba.ca/</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>Youth minor basketball; organizes coaching clinics and programs for the Southern Victoria area</t>
         </is>
       </c>
-      <c r="L31" t="inlineStr">
+      <c r="M31" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>WordPress (svba.ca)</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>primary</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
+      <c r="P31" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P31" t="inlineStr">
+      <c r="Q31" t="inlineStr">
         <is>
           <t>svba.ca returned HTTP 503 at time of check (2026-07-14) but is the club's registered site; Facebook page SVBasketballClub active.</t>
         </is>
@@ -2621,47 +2621,47 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Victoria County (BNB Central/West)</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Perth-Andover</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>https://svba.ca/</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>Youth basketball in the Perth-Andover area; fields 'Southern Victoria Vikings' teams in BNB youth divisions; uses River Valley Civic Centre (11 School St)</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>BNB Provincial League (U12-U14)</t>
         </is>
       </c>
-      <c r="L32" t="inlineStr">
+      <c r="M32" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t>reported</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
+      <c r="P32" t="inlineStr">
         <is>
           <t>https://svba.ca/</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
+      <c r="Q32" t="inlineStr">
         <is>
           <t>svba.ca returned HTTP 503 at check (Retry-After 1h) — site exists but was unavailable; registry lists club as 'Southern Victoria Basketball Club' with Facebook page facebook.com/SVBasketballClub.</t>
         </is>
@@ -2678,53 +2678,53 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Port Elgin</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>http://pemba.pointstreaksites.com/view/pemba/</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>Minor basketball; fielded 'Port Elgin Pirates' teams (incl. mini girls basketball) in NB Basketball Pointstreak-era seasons</t>
         </is>
       </c>
-      <c r="L33" t="inlineStr">
+      <c r="M33" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>Pointstreak Sites (legacy; site now redirects to stacksports.com)</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>uncertain</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
+      <c r="P33" t="inlineStr">
         <is>
           <t>http://pointstreak.com/players/players-team.html?teamid=358109&amp;seasonid=8295</t>
         </is>
       </c>
-      <c r="P33" t="inlineStr">
+      <c r="Q33" t="inlineStr">
         <is>
           <t>Likely dormant/defunct — website dead, not on current BNB registry. Evidence is legacy Pointstreak 'NB Basketball' pages; village (pop ~400) sits near Sackville. Verify existence before outreach.</t>
         </is>
-      </c>
-      <c r="Q33" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -2738,67 +2738,67 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Kennebecasis Valley</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Quispamsis/Rothesay</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>P.O. Box 4524, Rothesay, NB E2E 5X2</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>president@kvba.ca</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>https://kvba.ca/</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>Huey Lord, President (2025-26)</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>Winter house league + spring recreational (house) program U7, U9, U11, U14/U15, U18; competitive/rep program (Competitive Director role, repteams@kvba.ca); hosted BNB events</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>Kennebecasis Valley Basketball Association (KVBA) house league; BNB-sanctioned club tournament circuit (winter weekends); BNB Provincial League (U12-U14); BNB Provincial Championships U12/U13/U14</t>
         </is>
       </c>
-      <c r="L34" t="inlineStr">
+      <c r="M34" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>TeamSnap (registration); WordPress website</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr">
+      <c r="O34" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
+      <c r="P34" t="inlineStr">
         <is>
           <t>https://kvba.ca/</t>
         </is>
       </c>
-      <c r="P34" t="inlineStr">
+      <c r="Q34" t="inlineStr">
         <is>
           <t>2025-26 board fully published (VP Carrie Macfarlane, Treasurer Will MacEachern, Registrar Todd Potter, plus per-division house directors). Also has a SportsEngine org stub page.</t>
         </is>
@@ -2815,68 +2815,68 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" t="n">
+        <v>5</v>
+      </c>
+      <c r="D35" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Riverview</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>rmbaexec@gmail.com</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>https://www.rmba.ca/</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="J35" t="inlineStr">
         <is>
           <t>Amanda Lutes, President</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>Recreational community/house league boys &amp; girls ages 4-13; BNB Provincial Competitive rep teams (grades 4-8 tryouts); co-ed summer camp; 100% volunteer-run</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>Riverview Minor Basketball Association (RMBA) community league — operator; BNB Provincial League (U12-U14); BNB Provincial Championships U12/U13/U14; BNB U11 Kickoff (Nov) &amp; U11 Spring Finale (Feb); Moncton Basketball Association (MBA) recreational + spring leagues</t>
         </is>
       </c>
-      <c r="L35" t="inlineStr">
+      <c r="M35" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>RAMP InterActive (website, RAMP Registrations, RAMP Official Assigning)</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
+      <c r="P35" t="inlineStr">
         <is>
           <t>https://www.rmba.ca/</t>
         </is>
       </c>
-      <c r="P35" t="inlineStr">
+      <c r="Q35" t="inlineStr">
         <is>
           <t>Partners with MWBA Moncton Mystics (senior women) for community events. Only the president is published on the executives page.</t>
         </is>
-      </c>
-      <c r="Q35" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="36">
@@ -2890,52 +2890,52 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Greater Saint John / Kennebecasis Valley (BNB South)</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>Rothesay</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>surgebasketballacademy@hotmail.com</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>https://www.surgebasketball.com/</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>Elite/rep competitive teams — started girls-only with one team, now multiple girls and boys teams competing provincially and nationally; high-level coaching and individualized training; various age divisions up to U18</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>BNB-sanctioned club tournament circuit (winter weekends); BNB Provincial Championships U12/U13/U14; BNB U11 Kickoff (Nov) &amp; U11 Spring Finale (Feb)</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="M36" t="inlineStr">
         <is>
           <t>private academy (registered for-profit club)</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="O36" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
+      <c r="P36" t="inlineStr">
         <is>
           <t>https://www.surgebasketball.com/</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
+      <c r="Q36" t="inlineStr">
         <is>
           <t>Registered in Rothesay, described as 'elite basketball academy located in Saint John' — operates across greater Saint John/KV. Sponsored by GFL. Owner/founder name not published on site. | Also listed as: Surge Basketball</t>
         </is>
@@ -2952,47 +2952,47 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB (Municipality of Tantramar)</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>Sackville</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/928493714005177/</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>Youth basketball program in Sackville, NB (per Instagram bio); details published only via Facebook group / Instagram</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="M37" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>none found — Facebook group + Instagram only</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
+      <c r="O37" t="inlineStr">
         <is>
           <t>primary</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
+      <c r="P37" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P37" t="inlineStr">
+      <c r="Q37" t="inlineStr">
         <is>
           <t>CAUTION for pipeline dedup: 'Sackville Minor Basketball Association / Sackville Storm' (sackvillestorm.com, RAMP) is Lower Sackville, NOVA SCOTIA — not this club; verified via site's Lower Sackville weather widget and Sport NS raffle. Municipality of Tantramar also runs a free weekly youth basketball rec session at Dorchester Consolidated School (municipal program, not a club). | Community association; Basketball NB 2025-26 member, East Region (source: https://www.basketball.nb.ca/content/find-a-club-association). Web presence is Facebook group + Instagram @sbba_sackville_basketball (https://www.instagram.com/sbba_sackville_basketball/ — bio login-walled, could not extract email). No website, address, phone, or named executive found anywhere public. CAUTION: do not conflate with 'Sackville Minor Basketball Association / Sackville Storm' (sackvillestorm.com) — verified that org is Lower Sackville, NOVA SCOTIA. Town of Sackville rec dept 506-364-4958 is the only adjacent phone (municipal, not the club).</t>
         </is>
@@ -3009,57 +3009,57 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>Saint John area (BNB South Region)</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Saint John</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>40 College Hill Road, Rothesay, NB E2E 5H1</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>506-644-8479</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>damian.gay@rns.cc</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>https://www.rns.cc/camps/ecba</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>Damian Gay — founder/director (RNS teacher and Prep Boys basketball coach)</t>
         </is>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="M38" t="inlineStr">
         <is>
           <t>community nonprofit (assumed)</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
+      <c r="O38" t="inlineStr">
         <is>
           <t>uncertain</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr">
+      <c r="P38" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr">
+      <c r="Q38" t="inlineStr">
         <is>
           <t>On BNB 2025-26 member list (South Region) but no independent web presence found; exact home town unconfirmed. Do not confuse with East Coast Games (multi-sport event) or the US East Coast Basketball League. | IDENTITY CAVEAT: Basketball NB member list (South Region) says 'East Coast Basketball Association' with no link (https://www.basketball.nb.ca/content/find-a-club-association); the only ECBA in the Saint John region is 'East Coast Basketball Academy' — probable same entity but unconfirmed. Type: private academy (basketball-specific training company) run by Damian Gay out of Rothesay Netherwood School's Irving Gymnasium. Sources: Facebook page (https://www.facebook.com/eastcoastbasketballacademy/ — address, phone 506-644-8479, email damian.gay@rns.cc) and RNS page (https://www.rns.cc/camps/ecba — programs Junior Boys 9-12, Senior Boys 14-17, girls divisions; alt phone 506-847-8224; camps admin Geoffrey McCullogh 506-847-2619). COMPETITIVE INTEL: registration runs on TeamSnap (registration.teamsnap.com).</t>
         </is>
@@ -3076,57 +3076,57 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>Saint John (East)</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>Saint John</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>esjmbamike@gmail.com</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>https://esjmba.com/</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>Mike Roy, President (2024-25 board); Michael White, Vice-President</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>House league with age divisions from U7 up to U14+ (division heads listed for U7 and U14); inclusive program coordinator; officiating and events programs</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>East Saint John Minor Basketball Association house league</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="M39" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
+      <c r="O39" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr">
+      <c r="P39" t="inlineStr">
         <is>
           <t>https://esjmba.com/</t>
         </is>
       </c>
-      <c r="P39" t="inlineStr">
+      <c r="Q39" t="inlineStr">
         <is>
           <t>Full 15-person board published for 2024-25. Listed on City of Saint John local sport organizations directory.</t>
         </is>
@@ -3143,52 +3143,52 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>Saint John</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>Saint John</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>https://themwba.ca/teams/port-city-fog/</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>Paul Hickey, President (Port City Fog); Peter Hickey, General Manager</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>Girls spring development program created by the Port City Fog (Maritime Women's Basketball Association franchise) to link the franchise with the southern NB basketball community</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>BNB-sanctioned spring play (under Basketball NB umbrella)</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="M40" t="inlineStr">
         <is>
           <t>community program of semi-pro women's team (Port City Fog, MWBA)</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr">
+      <c r="O40" t="inlineStr">
         <is>
           <t>reported</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr">
+      <c r="P40" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr">
+      <c r="Q40" t="inlineStr">
         <is>
           <t>Listed as 'Jr. Fog' on BNB 2025-26 member list (South Region). Analogous to Fredericton's Jr. Freeze model. | Girls/junior program under the Port City Fog (Maritime Women's Basketball Association franchise); listed as its own Basketball NB 2025-26 member club, South Region (https://www.basketball.nb.ca/content/find-a-club-association) with no link/contact. Parent-org leadership per MWBA 2026 team page: Paul Hickey President, Peter Hickey GM, Dominic Laviolette head coach (https://themwba.ca/teams/port-city-fog/); CBC 2022 named Jillian Wilton as Fog franchise owner (https://www.cbc.ca/news/canada/new-brunswick/maritime-women-s-basketball-association-gears-up-for-may-tip-off-1.6357468) — ownership may have changed. No Jr. Fog-specific contact published; league-wide email mwba.league@gmail.com only. Principal left empty because Fog leadership is not confirmed as the junior program's principal.</t>
         </is>
@@ -3205,52 +3205,52 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>Greater Saint John (BNB South)</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>Saint John</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>portcityfog@gmail.com</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>https://themwba.ca/teams/port-city-fog/</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="J41" t="inlineStr">
         <is>
           <t>Paul Hickey, President</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>Girls youth basketball (high-school ages) run as the junior arm of the Port City Fog, Saint John's Maritime Women's Basketball Association team; one of three MWBA clubs offering youth programming</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="M41" t="inlineStr">
         <is>
           <t>community nonprofit (youth arm of MWBA semi-pro women's team)</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr">
+      <c r="O41" t="inlineStr">
         <is>
           <t>reported</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr">
+      <c r="P41" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr">
+      <c r="Q41" t="inlineStr">
         <is>
           <t>Listed as 'Jr. Fog' in BNB member registry (South region). Email shown is the parent Fog organization's. MWBA Fog head coach 2025: Dominic Laviolette (parent team, not necessarily Jr. program lead). | enriched 2026-07-18</t>
         </is>
@@ -3267,47 +3267,47 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>Saint John</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>Saint John</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/4191807610851414/</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>Registered not-for-profit youth basketball league founded summer 2021; spring season; multiple age divisions up to U18 (boys); all skill levels</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>K's Port City Basketball spring league (own)</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="M42" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr">
+      <c r="O42" t="inlineStr">
         <is>
           <t>primary</t>
         </is>
       </c>
-      <c r="O42" t="inlineStr">
+      <c r="P42" t="inlineStr">
         <is>
           <t>https://www.saintjohnsports.com/listing/ks-port-city-basketball/</t>
         </is>
       </c>
-      <c r="P42" t="inlineStr">
+      <c r="Q42" t="inlineStr">
         <is>
           <t>Operates mainly through Facebook group; listed as 'Competitive Program' in Saint John Sports Directory. | Registered not-for-profit youth basketball league founded summer 2021; 'all children regardless of skill level' mandate (source: https://www.saintjohnsports.com/listing/ks-port-city-basketball/). Basketball NB 2025-26 member, South Region; fields rep teams incl. U13 Boys on BNB RAMP league site (https://www.basketball.nb.ca/team/12977/3950/35624/346780). Also listed in City of Saint John P.R.O. Kids youth-org directory (https://saintjohn.ca/en/parks-and-recreation/pro-kids/youth-organizations). Facebook group is the only contact channel (login-walled); founder/president name not published anywhere found — 'K's' initial suggests founder but NOT identified, do not guess.</t>
         </is>
@@ -3324,73 +3324,73 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" t="n">
+        <v>8</v>
+      </c>
+      <c r="D43" t="inlineStr">
         <is>
           <t>Saint John West (BNB South)</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>Saint John</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>PO Box 27019, Saint John, NB E2M 5S8</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>lancasterminorbasketball@gmail.com</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>https://www.lancasterhoops.com/</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="J43" t="inlineStr">
         <is>
           <t>Jonathan Hillier, President</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>House league U5, U7, U9, U11, U13/U14 (equal play); 'LMBA Lynx' Competitive Travel program; Jr. NBA program; hosts annual 'Battle On The Bay' tournament (~500 competitive players from around the Maritimes)</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>Lancaster Minor Basketball Association house league; BNB Provincial Championships U12/U13/U14; BNB-sanctioned club tournament circuit (winter weekends); BNB U11 Kickoff (Nov) &amp; U11 Spring Finale (Feb)</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="M43" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t>TeamSnap (site footer 'Powered by TeamSnap')</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr">
+      <c r="O43" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O43" t="inlineStr">
+      <c r="P43" t="inlineStr">
         <is>
           <t>https://www.lancasterhoops.com/</t>
         </is>
       </c>
-      <c r="P43" t="inlineStr">
+      <c r="Q43" t="inlineStr">
         <is>
           <t>One of the two big Saint John community associations (west side). BNB member (South region). | enriched 2026-07-18</t>
         </is>
-      </c>
-      <c r="Q43" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="44">
@@ -3404,62 +3404,62 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>Moncton &amp; southeast NB (serves Salisbury + Petitcodiac)</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>Salisbury</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>info@salisburybasketball.ca</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>https://salisburybasketball.ca/</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="J44" t="inlineStr">
         <is>
           <t>Rob Campbell, President (last published executive list is 2021/22 — may be stale; VP Sarah Colwell; Jr NBA coordinator Marcy Keith)</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>Youth basketball ages 4-18: Jr. NBA program (grown to ~75 entrants per Canada Basketball article), house-level development, and competitive teams (U11, U12, U14, Bantam) with 'We Grow Champions' motto and Women in Sport initiative</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>Moncton Basketball Association (MBA) recreational + spring leagues; BNB Provincial Championships U12/U13/U14 (reported); BNB-sanctioned club tournament circuit (winter weekends)</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="M44" t="inlineStr">
         <is>
           <t>community nonprofit (est. 2015)</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="N44" t="inlineStr">
         <is>
           <t>WordPress website (site content stale — registration platform posted seasonally via social, not identified)</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr">
+      <c r="O44" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr">
+      <c r="P44" t="inlineStr">
         <is>
           <t>https://salisburybasketball.ca/</t>
         </is>
       </c>
-      <c r="P44" t="inlineStr">
+      <c r="Q44" t="inlineStr">
         <is>
           <t>Active BNB member (current registry) but own website last updated ~2021 — Facebook is the live channel. GTM signal: no modern registration software. | Also listed as: Salisbury Petitcodiac Minor Basketball Association</t>
         </is>
@@ -3476,42 +3476,42 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Charlotte County / southwestern NB</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>St. George</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>https://www.facebook.com/St.Georgebasketball/</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>Regional youth minor basketball for southwestern NB communities</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="M45" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr">
+      <c r="O45" t="inlineStr">
         <is>
           <t>uncertain</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr">
+      <c r="P45" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P45" t="inlineStr">
+      <c r="Q45" t="inlineStr">
         <is>
           <t>On BNB 2025-26 member list (South Region). 'St.George Basketball' Facebook page appears to be its public face; a legacy NBA find-a-place-to-play directory listed contact Terry Hatt (St. George) — unverified, directory now offline. Home base town inferred. | Community/regional minor association serving southwest NB (Charlotte County); Basketball NB 2025-26 member, South Region, listed with NO link/contact (https://www.basketball.nb.ca/content/find-a-club-association). DATA CORRECTION: the census Facebook link facebook.com/St.Georgebasketball belongs to St George Basketball in NSW, AUSTRALIA (about text references sgba.com.au; videos vs Camden Valley Wildfire) — remove it. Unverified stale lead from a defunct NBA-Canada directory (nba.ecrew.ca, now dead DNS): St. George basketball contact 'Terry Hatt, terry.hatt@connors.ca'; a Terry Hatt also appears as President of Fundy Minor Basketball Association on hometeamsonline (page now 403s) — same Fundy-region geography but unconfirmed and possibly years old; treat as lead only, not verified contact.</t>
         </is>
@@ -3528,53 +3528,53 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" t="n">
+        <v>5</v>
+      </c>
+      <c r="D46" t="inlineStr">
         <is>
           <t>Charlotte County</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>St. Stephen</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>https://www.facebook.com/groups/673711246067744/</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>Youth minor basketball; town Parks &amp; Rec separately runs summer basketball classes ages 7-17; U14 team appears in BNB competition</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="L46" t="inlineStr">
         <is>
           <t>BNB Provincial League (U12-U14)</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="M46" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr">
+      <c r="O46" t="inlineStr">
         <is>
           <t>primary</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr">
+      <c r="P46" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr">
+      <c r="Q46" t="inlineStr">
         <is>
           <t>Operates via Facebook group 'St. Stephen Basketball Association/SSBA'. St. Stephen is home of the world's oldest basketball court (heritage org 'Canada First Basketball Inc.' — not a club). | Community minor association; Basketball NB 2025-26 member, South Region, listed with NO link/contact (https://www.basketball.nb.ca/content/find-a-club-association). Facebook group (from census) is the only channel; login-walled. Not listed in the Municipal District of St. Stephen community resource directory (https://town.ststephen.nb.ca/community/community-resource-directory — checked, 55 orgs, no basketball club). Runs joint camps/events with McAdam Minor Basketball Association (per McAdam MBA Facebook page). Fields a U14 team in NB minor league play. Municipal rec dept (506-467-7700, info@chocolatetown.ca) runs separate intro basketball lessons — not the association. | Also listed as: St. Stephen Minor Basketball Association</t>
         </is>
-      </c>
-      <c r="Q46" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="47">
@@ -3588,73 +3588,73 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" t="n">
+        <v>6</v>
+      </c>
+      <c r="D47" t="inlineStr">
         <is>
           <t>Saint John area (Kings County)</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>Sussex</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>Sussex, NB E4E 3V7</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>(506) 433-9341</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>[email protected]</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>https://sussexbasketball.sportngin.com/</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t>Fundamentals-focused house program: Puppy, Jr Mini, Mini (4-on-4) and Bantam (5-on-5) levels with equal playing time</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="L47" t="inlineStr">
         <is>
           <t>Sussex Minor Basketball Association house program</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
+      <c r="M47" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="N47" t="inlineStr">
         <is>
           <t>SportsEngine (SportNgin SRM website + registration)</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr">
+      <c r="O47" t="inlineStr">
         <is>
           <t>verified</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr">
+      <c r="P47" t="inlineStr">
         <is>
           <t>https://sussexbasketball.sportngin.com/</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr">
+      <c r="Q47" t="inlineStr">
         <is>
           <t>Phone from SportsEngine org listing. | enriched 2026-07-18</t>
         </is>
-      </c>
-      <c r="Q47" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="48">
@@ -3668,37 +3668,37 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Carleton County</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>Woodstock</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>Competitive/elite youth basketball (name implies rep-level program for Carleton County)</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr">
+      <c r="M48" t="inlineStr">
         <is>
           <t>community rep program (assumed)</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr">
+      <c r="O48" t="inlineStr">
         <is>
           <t>uncertain</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr">
+      <c r="P48" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P48" t="inlineStr">
+      <c r="Q48" t="inlineStr">
         <is>
           <t>On BNB 2025-26 member list (Central/West Region); no independent web presence found; home town inferred from county name.</t>
         </is>
@@ -3715,52 +3715,52 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>Carleton County / Upper River Valley (BNB Central/West)</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>Woodstock</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>PO Box 4307, Woodstock, NB E7M 6B7</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>http://www.woodstockminorbasketball.com/</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>Runs the Woodstock Minor Basketball League (local youth league) promoting basketball in the greater Woodstock area; affiliated with Basketball NB, NBAABO (officials), School District 14 and the Town of Woodstock</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="L49" t="inlineStr">
         <is>
           <t>BNB Provincial League (U12-U14); Woodstock Minor Basketball League (own house league)</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="M49" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr">
+      <c r="O49" t="inlineStr">
         <is>
           <t>reported</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr">
+      <c r="P49" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P49" t="inlineStr">
+      <c r="Q49" t="inlineStr">
         <is>
           <t>woodstockminorbasketball.com DNS did not resolve at check (site likely lapsed); Facebook page active; BNB registry links a facebook.com/share URL.</t>
         </is>
@@ -3777,27 +3777,27 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>Acadian Peninsula / BNB North Region (town unconfirmed)</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr">
+      <c r="M50" t="inlineStr">
         <is>
           <t>community nonprofit (assumed; francophone)</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr">
+      <c r="O50" t="inlineStr">
         <is>
           <t>uncertain</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr">
+      <c r="P50" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P50" t="inlineStr">
+      <c r="Q50" t="inlineStr">
         <is>
           <t>On BNB 2025-26 member list (North Region). French and English searches (Tracadie, Caraquet, Shippagan, Néguac) found no independent web presence. Likely serves the francophone Acadian Peninsula; Tracadie hosts Jeux de l'Acadie 2027 which includes youth basketball. No youth basketball club found in Campbellton/Restigouche — BNB North Region has only 3 members (Miramichi, Acadie, Bathurst).</t>
         </is>
@@ -3814,22 +3814,22 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>Carleton County / Upper River Valley (BNB Central/West)</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr">
+      <c r="O51" t="inlineStr">
         <is>
           <t>uncertain</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr">
+      <c r="P51" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr">
+      <c r="Q51" t="inlineStr">
         <is>
           <t>BNB 2025-26 registry entry only; name suggests a Carleton County rep/select program (likely Woodstock-based) but no independent evidence found.</t>
         </is>
@@ -3846,27 +3846,27 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>BNB Central/West Region (town unconfirmed)</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr">
+      <c r="M52" t="inlineStr">
         <is>
           <t>private academy (assumed from name)</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr">
+      <c r="O52" t="inlineStr">
         <is>
           <t>uncertain</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr">
+      <c r="P52" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P52" t="inlineStr">
+      <c r="Q52" t="inlineStr">
         <is>
           <t>On BNB 2025-26 member list (Central/West Region). No NB web presence found — do NOT confuse with eaglesbasketballacademy.com (Cochrane, Alberta). A Facebook page 'Eagles Academy' (EaglesAcademy001) may be related but unconfirmed. | Also listed as: Eagles Basketball Academy</t>
         </is>
@@ -3883,22 +3883,22 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>BNB South region (Greater Saint John area, exact town unconfirmed)</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr">
+      <c r="O53" t="inlineStr">
         <is>
           <t>uncertain</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr">
+      <c r="P53" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr">
+      <c r="Q53" t="inlineStr">
         <is>
           <t>Appears only on the BNB 2025-26 member registry (South region). No website, social page, or news coverage found; do not confuse with the pro ECBL league or East Coast orgs in NS.</t>
         </is>
@@ -3915,27 +3915,27 @@
           <t>New Brunswick</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>Charlotte County / southwest NB (BNB South)</t>
         </is>
       </c>
-      <c r="L54" t="inlineStr">
+      <c r="M54" t="inlineStr">
         <is>
           <t>community nonprofit</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr">
+      <c r="O54" t="inlineStr">
         <is>
           <t>uncertain</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr">
+      <c r="P54" t="inlineStr">
         <is>
           <t>https://www.basketball.nb.ca/content/find-a-club-association</t>
         </is>
       </c>
-      <c r="P54" t="inlineStr">
+      <c r="Q54" t="inlineStr">
         <is>
           <t>BNB 2025-26 member registry entry only (South region); likely serves the St. George/Blacks Harbour corridor but no independent web presence found — exact base town unconfirmed.</t>
         </is>

</xml_diff>